<commit_message>
Add about and user guide pages, enhance log filtering, and improve GTFS handling
- Created 'about.html' and 'userguide.html' templates with navigation.
- Updated 'index.html' to include links to the new pages.
- Enhanced 'log.html' with filtering options for search logs.
- Added JavaScript functionality for dynamic filtering of log entries.
- Improved the handling of GTFS data in 'views.py' to refresh the cache of stop names.
- Updated form placeholders in 'form.html' for better user guidance.
- Adjusted CSS styles in 'customstyle.css' for new UI elements.
</commit_message>
<xml_diff>
--- a/myapp/static/data/log/search_log.xlsx
+++ b/myapp/static/data/log/search_log.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="history" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="history" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S17"/>
+  <dimension ref="A1:S83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1713,6 +1713,4956 @@
         <v>39.3222</v>
       </c>
     </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026-05-21 17:18:50</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>17:16:00</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N18" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="O18" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="P18" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q18" t="n">
+        <v>0</v>
+      </c>
+      <c r="R18" t="n">
+        <v>0.0562</v>
+      </c>
+      <c r="S18" t="n">
+        <v>109.5426</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026-05-21 17:44:56</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>PIK Avenue</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>17:35:00</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N19" t="n">
+        <v>547</v>
+      </c>
+      <c r="O19" t="n">
+        <v>101.72</v>
+      </c>
+      <c r="P19" t="n">
+        <v>24500</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>25</v>
+      </c>
+      <c r="R19" t="n">
+        <v>2.7398</v>
+      </c>
+      <c r="S19" t="n">
+        <v>567.428</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2026-05-21 17:51:12</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>PIK Avenue</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>17:39:00</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J20" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L20" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M20" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N20" t="n">
+        <v>336.9</v>
+      </c>
+      <c r="O20" t="n">
+        <v>60.38</v>
+      </c>
+      <c r="P20" t="n">
+        <v>27000</v>
+      </c>
+      <c r="Q20" t="n">
+        <v>10</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1.7691</v>
+      </c>
+      <c r="S20" t="n">
+        <v>668.8851</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:56:35</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J21" t="n">
+        <v>25</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L21" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M21" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N21" t="n">
+        <v>123.3</v>
+      </c>
+      <c r="O21" t="n">
+        <v>34.27</v>
+      </c>
+      <c r="P21" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>5</v>
+      </c>
+      <c r="R21" t="n">
+        <v>0.5475</v>
+      </c>
+      <c r="S21" t="n">
+        <v>290.0624</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:57:53</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J22" t="n">
+        <v>25</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L22" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M22" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N22" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="O22" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="P22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="S22" t="n">
+        <v>32.6514</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-05-21 18:58:52</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>25</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L23" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M23" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N23" t="n">
+        <v>58.8</v>
+      </c>
+      <c r="O23" t="n">
+        <v>18.11</v>
+      </c>
+      <c r="P23" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>2</v>
+      </c>
+      <c r="R23" t="n">
+        <v>0.2211</v>
+      </c>
+      <c r="S23" t="n">
+        <v>48.6927</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-05-21 19:00:25</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>16:51:00</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>25</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M24" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N24" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="O24" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="P24" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="S24" t="n">
+        <v>46.4544</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-05-21 22:22:19</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Ragunan</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Tanjung Priok</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>25</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L25" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M25" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N25" t="n">
+        <v>260.6</v>
+      </c>
+      <c r="O25" t="n">
+        <v>89.7</v>
+      </c>
+      <c r="P25" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>6</v>
+      </c>
+      <c r="R25" t="n">
+        <v>0.7079</v>
+      </c>
+      <c r="S25" t="n">
+        <v>64.0462</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026-05-22 02:13:21</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Univ. Tarumanegara</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>min_transit</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J26" t="n">
+        <v>25</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M26" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N26" t="n">
+        <v>169.6</v>
+      </c>
+      <c r="O26" t="n">
+        <v>61.41</v>
+      </c>
+      <c r="P26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>4</v>
+      </c>
+      <c r="R26" t="n">
+        <v>0.6971000000000001</v>
+      </c>
+      <c r="S26" t="n">
+        <v>44.1984</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026-05-22 07:29:07</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>07:26:00</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J27" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N27" t="n">
+        <v>155</v>
+      </c>
+      <c r="O27" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="P27" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>2</v>
+      </c>
+      <c r="R27" t="n">
+        <v>0.3102</v>
+      </c>
+      <c r="S27" t="n">
+        <v>8.6731</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:26:39</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Harmoni</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J28" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L28" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M28" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N28" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="O28" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="P28" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="n">
+        <v>0.0669</v>
+      </c>
+      <c r="S28" t="n">
+        <v>14.8017</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:26:43</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Harmoni</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J29" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L29" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M29" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N29" t="n">
+        <v>36.2</v>
+      </c>
+      <c r="O29" t="n">
+        <v>10.57</v>
+      </c>
+      <c r="P29" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q29" t="n">
+        <v>0</v>
+      </c>
+      <c r="R29" t="n">
+        <v>0.0669</v>
+      </c>
+      <c r="S29" t="n">
+        <v>4.0445</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:29:36</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>08:28:00</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L30" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M30" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N30" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="O30" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P30" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q30" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" t="n">
+        <v>0.0556</v>
+      </c>
+      <c r="S30" t="n">
+        <v>17.4646</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:29:41</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>08:28:00</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M31" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N31" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="O31" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P31" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="n">
+        <v>0.0556</v>
+      </c>
+      <c r="S31" t="n">
+        <v>4.6899</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:33:00</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Harmoni</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>08:00:00</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L32" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M32" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N32" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="O32" t="n">
+        <v>23.26</v>
+      </c>
+      <c r="P32" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>5</v>
+      </c>
+      <c r="R32" t="n">
+        <v>0.4679</v>
+      </c>
+      <c r="S32" t="n">
+        <v>376.7314</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-05-22 08:35:12</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>08:28:00</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>JAM SIBUK</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L33" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M33" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N33" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="O33" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P33" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="n">
+        <v>0.0556</v>
+      </c>
+      <c r="S33" t="n">
+        <v>330.796</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-05-22 10:48:08</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PIK Avenue</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Bundaran Alam Sutera 1</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>2026-05-22</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>10:47:00</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>25</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L34" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M34" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N34" t="n">
+        <v>111</v>
+      </c>
+      <c r="O34" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="P34" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>1</v>
+      </c>
+      <c r="R34" t="n">
+        <v>0.2694</v>
+      </c>
+      <c r="S34" t="n">
+        <v>30.1958</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:42:28</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>25</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L35" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M35" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N35" t="n">
+        <v>1096</v>
+      </c>
+      <c r="O35" t="n">
+        <v>378.94</v>
+      </c>
+      <c r="P35" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>23</v>
+      </c>
+      <c r="R35" t="n">
+        <v>2.7482</v>
+      </c>
+      <c r="S35" t="n">
+        <v>23.2387</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:43:15</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>25</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L36" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M36" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N36" t="n">
+        <v>1289.2</v>
+      </c>
+      <c r="O36" t="n">
+        <v>458.92</v>
+      </c>
+      <c r="P36" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q36" t="n">
+        <v>27</v>
+      </c>
+      <c r="R36" t="n">
+        <v>3.1937</v>
+      </c>
+      <c r="S36" t="n">
+        <v>29.4569</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:44:32</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>25</v>
+      </c>
+      <c r="K37" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L37" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M37" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N37" t="n">
+        <v>491.4</v>
+      </c>
+      <c r="O37" t="n">
+        <v>177.5</v>
+      </c>
+      <c r="P37" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>10</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1.2217</v>
+      </c>
+      <c r="S37" t="n">
+        <v>23.1354</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:45:55</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>25</v>
+      </c>
+      <c r="K38" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L38" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M38" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N38" t="n">
+        <v>566.9</v>
+      </c>
+      <c r="O38" t="n">
+        <v>164.38</v>
+      </c>
+      <c r="P38" t="n">
+        <v>14000</v>
+      </c>
+      <c r="Q38" t="n">
+        <v>16</v>
+      </c>
+      <c r="R38" t="n">
+        <v>1.8582</v>
+      </c>
+      <c r="S38" t="n">
+        <v>19.1568</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:46:40</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>25</v>
+      </c>
+      <c r="K39" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L39" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M39" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N39" t="n">
+        <v>227.8</v>
+      </c>
+      <c r="O39" t="n">
+        <v>72.93000000000001</v>
+      </c>
+      <c r="P39" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>4</v>
+      </c>
+      <c r="R39" t="n">
+        <v>0.6776</v>
+      </c>
+      <c r="S39" t="n">
+        <v>18.3199</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:48:38</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>25</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L40" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M40" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N40" t="n">
+        <v>1348.4</v>
+      </c>
+      <c r="O40" t="n">
+        <v>461.31</v>
+      </c>
+      <c r="P40" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>33</v>
+      </c>
+      <c r="R40" t="n">
+        <v>3.7152</v>
+      </c>
+      <c r="S40" t="n">
+        <v>25.5067</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:51:53</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>25</v>
+      </c>
+      <c r="K41" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L41" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M41" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N41" t="n">
+        <v>274.5</v>
+      </c>
+      <c r="O41" t="n">
+        <v>72.43000000000001</v>
+      </c>
+      <c r="P41" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>11</v>
+      </c>
+      <c r="R41" t="n">
+        <v>1.2875</v>
+      </c>
+      <c r="S41" t="n">
+        <v>101.7261</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:54:44</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>25</v>
+      </c>
+      <c r="K42" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L42" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M42" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N42" t="n">
+        <v>576</v>
+      </c>
+      <c r="O42" t="n">
+        <v>198.41</v>
+      </c>
+      <c r="P42" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>15</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.6333</v>
+      </c>
+      <c r="S42" t="n">
+        <v>55.3172</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:56:36</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>25</v>
+      </c>
+      <c r="K43" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L43" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M43" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N43" t="n">
+        <v>440.9</v>
+      </c>
+      <c r="O43" t="n">
+        <v>158.91</v>
+      </c>
+      <c r="P43" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>9</v>
+      </c>
+      <c r="R43" t="n">
+        <v>1.1749</v>
+      </c>
+      <c r="S43" t="n">
+        <v>57.1999</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:57:59</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>25</v>
+      </c>
+      <c r="K44" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L44" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M44" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N44" t="n">
+        <v>893</v>
+      </c>
+      <c r="O44" t="n">
+        <v>292.34</v>
+      </c>
+      <c r="P44" t="n">
+        <v>17500</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>19</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.4601</v>
+      </c>
+      <c r="S44" t="n">
+        <v>49.2174</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2026-05-22 12:58:44</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>25</v>
+      </c>
+      <c r="K45" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L45" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M45" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N45" t="n">
+        <v>544.7</v>
+      </c>
+      <c r="O45" t="n">
+        <v>177.43</v>
+      </c>
+      <c r="P45" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>15</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.6043</v>
+      </c>
+      <c r="S45" t="n">
+        <v>32.3689</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:01:22</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>25</v>
+      </c>
+      <c r="K46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M46" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N46" t="n">
+        <v>1120.5</v>
+      </c>
+      <c r="O46" t="n">
+        <v>378.09</v>
+      </c>
+      <c r="P46" t="n">
+        <v>31500</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>25</v>
+      </c>
+      <c r="R46" t="n">
+        <v>3.0708</v>
+      </c>
+      <c r="S46" t="n">
+        <v>81.99939999999999</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:17:39</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>25</v>
+      </c>
+      <c r="K47" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L47" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M47" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N47" t="n">
+        <v>753.8</v>
+      </c>
+      <c r="O47" t="n">
+        <v>264.27</v>
+      </c>
+      <c r="P47" t="n">
+        <v>17500</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>17</v>
+      </c>
+      <c r="R47" t="n">
+        <v>1.998</v>
+      </c>
+      <c r="S47" t="n">
+        <v>69.26300000000001</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:25:07</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>25</v>
+      </c>
+      <c r="K48" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L48" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M48" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N48" t="n">
+        <v>1251.3</v>
+      </c>
+      <c r="O48" t="n">
+        <v>278.96</v>
+      </c>
+      <c r="P48" t="n">
+        <v>38500</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>73</v>
+      </c>
+      <c r="R48" t="n">
+        <v>7.392</v>
+      </c>
+      <c r="S48" t="n">
+        <v>28.9999</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:26:05</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>25</v>
+      </c>
+      <c r="K49" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L49" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M49" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N49" t="n">
+        <v>1462.3</v>
+      </c>
+      <c r="O49" t="n">
+        <v>285.4</v>
+      </c>
+      <c r="P49" t="n">
+        <v>66500</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>88</v>
+      </c>
+      <c r="R49" t="n">
+        <v>9.120699999999999</v>
+      </c>
+      <c r="S49" t="n">
+        <v>29.3728</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:29:47</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>25</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M50" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N50" t="n">
+        <v>392.7</v>
+      </c>
+      <c r="O50" t="n">
+        <v>113.02</v>
+      </c>
+      <c r="P50" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>12</v>
+      </c>
+      <c r="R50" t="n">
+        <v>1.4637</v>
+      </c>
+      <c r="S50" t="n">
+        <v>69.0065</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:32:20</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>25</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M51" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N51" t="n">
+        <v>921.3</v>
+      </c>
+      <c r="O51" t="n">
+        <v>255.28</v>
+      </c>
+      <c r="P51" t="n">
+        <v>31500</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>38</v>
+      </c>
+      <c r="R51" t="n">
+        <v>3.8864</v>
+      </c>
+      <c r="S51" t="n">
+        <v>79.98390000000001</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:35:02</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>25</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M52" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N52" t="n">
+        <v>1240.7</v>
+      </c>
+      <c r="O52" t="n">
+        <v>445.83</v>
+      </c>
+      <c r="P52" t="n">
+        <v>21000</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>27</v>
+      </c>
+      <c r="R52" t="n">
+        <v>3.1488</v>
+      </c>
+      <c r="S52" t="n">
+        <v>148.4716</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:39:52</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>25</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M53" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N53" t="n">
+        <v>504.1</v>
+      </c>
+      <c r="O53" t="n">
+        <v>182.99</v>
+      </c>
+      <c r="P53" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>11</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1.2667</v>
+      </c>
+      <c r="S53" t="n">
+        <v>64.54989999999999</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:41:37</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>25</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M54" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N54" t="n">
+        <v>262.4</v>
+      </c>
+      <c r="O54" t="n">
+        <v>93.13</v>
+      </c>
+      <c r="P54" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>5</v>
+      </c>
+      <c r="R54" t="n">
+        <v>0.643</v>
+      </c>
+      <c r="S54" t="n">
+        <v>81.3429</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:47:05</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>25</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M55" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N55" t="n">
+        <v>500.2</v>
+      </c>
+      <c r="O55" t="n">
+        <v>177.3</v>
+      </c>
+      <c r="P55" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>8</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1.0965</v>
+      </c>
+      <c r="S55" t="n">
+        <v>39.4789</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:48:46</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>25</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M56" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N56" t="n">
+        <v>383.6</v>
+      </c>
+      <c r="O56" t="n">
+        <v>133.94</v>
+      </c>
+      <c r="P56" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>10</v>
+      </c>
+      <c r="R56" t="n">
+        <v>1.0885</v>
+      </c>
+      <c r="S56" t="n">
+        <v>74.0889</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:50:31</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>25</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M57" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N57" t="n">
+        <v>486.3</v>
+      </c>
+      <c r="O57" t="n">
+        <v>176.84</v>
+      </c>
+      <c r="P57" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>10</v>
+      </c>
+      <c r="R57" t="n">
+        <v>1.1836</v>
+      </c>
+      <c r="S57" t="n">
+        <v>82.4954</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>2026-05-22 13:53:29</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>25</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M58" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N58" t="n">
+        <v>308.8</v>
+      </c>
+      <c r="O58" t="n">
+        <v>108.6</v>
+      </c>
+      <c r="P58" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>6</v>
+      </c>
+      <c r="R58" t="n">
+        <v>0.7526</v>
+      </c>
+      <c r="S58" t="n">
+        <v>144.3914</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:02:15</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>25</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M59" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N59" t="n">
+        <v>148.1</v>
+      </c>
+      <c r="O59" t="n">
+        <v>51.36</v>
+      </c>
+      <c r="P59" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>3</v>
+      </c>
+      <c r="R59" t="n">
+        <v>0.4038</v>
+      </c>
+      <c r="S59" t="n">
+        <v>84.3558</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:02:15</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>25</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M60" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N60" t="n">
+        <v>142</v>
+      </c>
+      <c r="O60" t="n">
+        <v>48.24</v>
+      </c>
+      <c r="P60" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>4</v>
+      </c>
+      <c r="R60" t="n">
+        <v>0.4649</v>
+      </c>
+      <c r="S60" t="n">
+        <v>62.6521</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:04:33</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>25</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M61" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N61" t="n">
+        <v>126.4</v>
+      </c>
+      <c r="O61" t="n">
+        <v>45.08</v>
+      </c>
+      <c r="P61" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>3</v>
+      </c>
+      <c r="R61" t="n">
+        <v>0.3837</v>
+      </c>
+      <c r="S61" t="n">
+        <v>79.87050000000001</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:06:42</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>25</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M62" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N62" t="n">
+        <v>221.6</v>
+      </c>
+      <c r="O62" t="n">
+        <v>76.64</v>
+      </c>
+      <c r="P62" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>4</v>
+      </c>
+      <c r="R62" t="n">
+        <v>0.5385</v>
+      </c>
+      <c r="S62" t="n">
+        <v>74.018</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:08:52</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>25</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M63" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N63" t="n">
+        <v>350</v>
+      </c>
+      <c r="O63" t="n">
+        <v>112.86</v>
+      </c>
+      <c r="P63" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>9</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1.0241</v>
+      </c>
+      <c r="S63" t="n">
+        <v>22.557</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:09:27</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>25</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M64" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N64" t="n">
+        <v>345.7</v>
+      </c>
+      <c r="O64" t="n">
+        <v>125.48</v>
+      </c>
+      <c r="P64" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>7</v>
+      </c>
+      <c r="R64" t="n">
+        <v>0.8534</v>
+      </c>
+      <c r="S64" t="n">
+        <v>18.7175</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:10:50</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>25</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M65" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N65" t="n">
+        <v>330.9</v>
+      </c>
+      <c r="O65" t="n">
+        <v>108.83</v>
+      </c>
+      <c r="P65" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>9</v>
+      </c>
+      <c r="R65" t="n">
+        <v>0.9731</v>
+      </c>
+      <c r="S65" t="n">
+        <v>51.3042</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:12:54</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>25</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M66" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N66" t="n">
+        <v>308.8</v>
+      </c>
+      <c r="O66" t="n">
+        <v>110.72</v>
+      </c>
+      <c r="P66" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>7</v>
+      </c>
+      <c r="R66" t="n">
+        <v>0.8192</v>
+      </c>
+      <c r="S66" t="n">
+        <v>79.8837</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:17:22</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>25</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M67" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N67" t="n">
+        <v>455.8</v>
+      </c>
+      <c r="O67" t="n">
+        <v>146.33</v>
+      </c>
+      <c r="P67" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>11</v>
+      </c>
+      <c r="R67" t="n">
+        <v>1.322</v>
+      </c>
+      <c r="S67" t="n">
+        <v>144.8382</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:34:36</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>25</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M68" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N68" t="n">
+        <v>165.4</v>
+      </c>
+      <c r="O68" t="n">
+        <v>52.15</v>
+      </c>
+      <c r="P68" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>3</v>
+      </c>
+      <c r="R68" t="n">
+        <v>0.4865</v>
+      </c>
+      <c r="S68" t="n">
+        <v>100.2409</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:36:31</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>25</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M69" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N69" t="n">
+        <v>154.9</v>
+      </c>
+      <c r="O69" t="n">
+        <v>52.76</v>
+      </c>
+      <c r="P69" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>4</v>
+      </c>
+      <c r="R69" t="n">
+        <v>0.4767</v>
+      </c>
+      <c r="S69" t="n">
+        <v>89.6923</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:39:17</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>25</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M70" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N70" t="n">
+        <v>823.5</v>
+      </c>
+      <c r="O70" t="n">
+        <v>208.17</v>
+      </c>
+      <c r="P70" t="n">
+        <v>42000</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>40</v>
+      </c>
+      <c r="R70" t="n">
+        <v>4.4292</v>
+      </c>
+      <c r="S70" t="n">
+        <v>125.4554</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:45:22</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>25</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M71" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N71" t="n">
+        <v>168.6</v>
+      </c>
+      <c r="O71" t="n">
+        <v>56.67</v>
+      </c>
+      <c r="P71" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>4</v>
+      </c>
+      <c r="R71" t="n">
+        <v>0.5561</v>
+      </c>
+      <c r="S71" t="n">
+        <v>162.9118</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-05-22 14:49:20</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>25</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M72" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N72" t="n">
+        <v>237.4</v>
+      </c>
+      <c r="O72" t="n">
+        <v>84.27</v>
+      </c>
+      <c r="P72" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>5</v>
+      </c>
+      <c r="R72" t="n">
+        <v>0.6199</v>
+      </c>
+      <c r="S72" t="n">
+        <v>110.2599</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-05-22 15:15:21</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>25</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M73" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N73" t="n">
+        <v>210.4</v>
+      </c>
+      <c r="O73" t="n">
+        <v>70.23</v>
+      </c>
+      <c r="P73" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>5</v>
+      </c>
+      <c r="R73" t="n">
+        <v>0.6948</v>
+      </c>
+      <c r="S73" t="n">
+        <v>78.6377</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-05-23 09:20:01</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>25</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M74" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N74" t="n">
+        <v>203.8</v>
+      </c>
+      <c r="O74" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="P74" t="n">
+        <v>10500</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>6</v>
+      </c>
+      <c r="R74" t="n">
+        <v>0.6887</v>
+      </c>
+      <c r="S74" t="n">
+        <v>84.3841</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:30:40</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>02:30:00</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>40</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M75" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N75" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="O75" t="n">
+        <v>7.22</v>
+      </c>
+      <c r="P75" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" t="n">
+        <v>0.0434</v>
+      </c>
+      <c r="S75" t="n">
+        <v>4.7774</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:30:52</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>02:30:00</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>40</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M76" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N76" t="n">
+        <v>106.6</v>
+      </c>
+      <c r="O76" t="n">
+        <v>51.16</v>
+      </c>
+      <c r="P76" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>5</v>
+      </c>
+      <c r="R76" t="n">
+        <v>0.4653</v>
+      </c>
+      <c r="S76" t="n">
+        <v>6.8968</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:33:47</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>02:32:00</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>HACO</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>40</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M77" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N77" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="O77" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P77" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="S77" t="n">
+        <v>73.65049999999999</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:35:08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Grogol</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>02:32:00</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>40</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M78" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N78" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="O78" t="n">
+        <v>14.85</v>
+      </c>
+      <c r="P78" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>1</v>
+      </c>
+      <c r="R78" t="n">
+        <v>0.1234</v>
+      </c>
+      <c r="S78" t="n">
+        <v>8.5633</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:42:39</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>02:39:00</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>40</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M79" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N79" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="O79" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P79" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" t="n">
+        <v>0.0431</v>
+      </c>
+      <c r="S79" t="n">
+        <v>13.6565</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>2026-05-24 02:52:43</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Bundaran HI Astra</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Blok M</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>02:39:00</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>seimbang</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>MILP</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>JAM MALAM</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>40</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="M80" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="N80" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="O80" t="n">
+        <v>7.03</v>
+      </c>
+      <c r="P80" t="n">
+        <v>3500</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>0.0446</v>
+      </c>
+      <c r="S80" t="n">
+        <v>8.4495</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:47:49</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>min_transit</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>25</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M81" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N81" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="O81" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="P81" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>2</v>
+      </c>
+      <c r="R81" t="n">
+        <v>0.3743</v>
+      </c>
+      <c r="S81" t="n">
+        <v>2.2907</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>2026-05-25 17:48:20</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>min_transit</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>25</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M82" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N82" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="O82" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="P82" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>2</v>
+      </c>
+      <c r="R82" t="n">
+        <v>0.3743</v>
+      </c>
+      <c r="S82" t="n">
+        <v>2.2185</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>2026-05-25 18:01:00</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Kalideres</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Pulo Gebang</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>min_transit</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>ASTAR</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>JAM NORMAL</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>25</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="M83" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="N83" t="n">
+        <v>123.6</v>
+      </c>
+      <c r="O83" t="n">
+        <v>41.26</v>
+      </c>
+      <c r="P83" t="n">
+        <v>7000</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>2</v>
+      </c>
+      <c r="R83" t="n">
+        <v>0.3743</v>
+      </c>
+      <c r="S83" t="n">
+        <v>2.1717</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>